<commit_message>
Set Dont and No Compromise text to 16pt
</commit_message>
<xml_diff>
--- a/templates/template_general.xlsx
+++ b/templates/template_general.xlsx
@@ -5,174 +5,282 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Bot\Market_Survey_Git\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Bot\Market_Survey\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55D7F885-6DDF-4E5D-8747-A16E5D0768AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B25F2DF4-1F0D-49D1-80B7-A9070E8BC248}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Simaple_form" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Simaple_form!$A$1:$AA$48</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="92">
   <si>
     <t>Market Improvement Report</t>
   </si>
   <si>
+    <t>PRODUCT FRESHNESS, AVAILIBILITY &amp; NEW OUTLET LIST IN</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <t>BBE</t>
+  </si>
+  <si>
+    <t>Wholesale: 0</t>
+  </si>
+  <si>
+    <t>Drink Shop: 19</t>
+  </si>
+  <si>
+    <t>Wet Market: 0</t>
+  </si>
+  <si>
+    <t>Trolley: 10</t>
+  </si>
+  <si>
+    <t>New Outlet Purchase</t>
+  </si>
+  <si>
+    <t>Volume</t>
+  </si>
+  <si>
+    <t>CB LITE ORD</t>
+  </si>
+  <si>
+    <t>CBC 4.4 NCP</t>
+  </si>
+  <si>
+    <t>CB Original NCP</t>
+  </si>
+  <si>
+    <t>CB LITE NCP</t>
+  </si>
+  <si>
+    <t>CB BLACK NCP</t>
+  </si>
+  <si>
+    <t>CAMBODIA COLA</t>
+  </si>
+  <si>
+    <t>CAMBODIA ED</t>
+  </si>
+  <si>
+    <t>IZE PET 300ml Flavour</t>
+  </si>
+  <si>
+    <t>IZE COLA PET 1.5L All SKUs</t>
+  </si>
+  <si>
+    <t>CAMBODIA WATER 500mL</t>
+  </si>
+  <si>
+    <t>CAMBODIA WATER 1500mL</t>
+  </si>
+  <si>
+    <t>PRODUCT MOVEMENT VS COMPETITOR</t>
+  </si>
+  <si>
+    <t>#</t>
+  </si>
+  <si>
+    <t>Mov</t>
+  </si>
+  <si>
+    <t>Stock</t>
+  </si>
+  <si>
+    <t>Buy In</t>
+  </si>
+  <si>
+    <t>Sell Out</t>
+  </si>
+  <si>
+    <t>Ring Pull</t>
+  </si>
+  <si>
+    <t>GB SNOW ORD</t>
+  </si>
+  <si>
+    <t>HANUMAN LITE ORD</t>
+  </si>
+  <si>
+    <t>Krud LITE ORD</t>
+  </si>
+  <si>
+    <t>GB Original NCP</t>
+  </si>
+  <si>
+    <t>Krud NCP</t>
+  </si>
+  <si>
+    <t>GB SNOW NCP</t>
+  </si>
+  <si>
+    <t>Hanuman LITE NCP</t>
+  </si>
+  <si>
+    <t>Krud LITE NCP</t>
+  </si>
+  <si>
+    <t>Greet LITE NCP</t>
+  </si>
+  <si>
+    <t>Hanuman Black NCP</t>
+  </si>
+  <si>
+    <t>CAMBODIA COLA 330ml</t>
+  </si>
+  <si>
+    <t>Coca Cola 330ml</t>
+  </si>
+  <si>
+    <t>BACCHUSE Sugar Free</t>
+  </si>
+  <si>
+    <t>IZE PET 300ml All SKUs</t>
+  </si>
+  <si>
+    <t>POP Z Flavour</t>
+  </si>
+  <si>
+    <t>V Cola 350ml</t>
+  </si>
+  <si>
+    <t>Coca 1.5L</t>
+  </si>
+  <si>
+    <t>Big Cola 3L</t>
+  </si>
+  <si>
+    <t>Sting Can 330ml</t>
+  </si>
+  <si>
+    <t>Pocari Sweat</t>
+  </si>
+  <si>
+    <t>V-Active Sport</t>
+  </si>
+  <si>
+    <t>Vital 500mL</t>
+  </si>
+  <si>
+    <t>Provida 500mL</t>
+  </si>
+  <si>
+    <t>Ganzberg 500ml</t>
+  </si>
+  <si>
+    <t>Hitech 500mL</t>
+  </si>
+  <si>
+    <t>Vital 1500mL</t>
+  </si>
+  <si>
+    <t>Provida 1500mL</t>
+  </si>
+  <si>
+    <t>Ganzberg 1500ml</t>
+  </si>
+  <si>
+    <t>Hitech 1500mL</t>
+  </si>
+  <si>
+    <t>2.</t>
+  </si>
+  <si>
+    <t>3.</t>
+  </si>
+  <si>
+    <t>4.</t>
+  </si>
+  <si>
+    <t>Location of Visit:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Group : </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Member : </t>
+  </si>
+  <si>
+    <t>Total outlet Visit :</t>
+  </si>
+  <si>
     <t>Dealer :                                                      Report Date:</t>
   </si>
   <si>
-    <t xml:space="preserve">Group : </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Member : </t>
-  </si>
-  <si>
-    <t>Location of Visit:</t>
-  </si>
-  <si>
-    <t>Total outlet Visit :</t>
-  </si>
-  <si>
-    <t>PRODUCT FRESHNESS, AVAILIBILITY &amp; NEW OUTLET LIST IN</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Product</t>
-  </si>
-  <si>
-    <t>BBE</t>
-  </si>
-  <si>
-    <t>Wholesale: 0</t>
-  </si>
-  <si>
-    <t>Drink Shop: 19</t>
-  </si>
-  <si>
-    <t>Wet Market: 0</t>
-  </si>
-  <si>
-    <t>Trolley: 10</t>
-  </si>
-  <si>
-    <t>New Outlet Purchase</t>
-  </si>
-  <si>
-    <t>Volume</t>
-  </si>
-  <si>
-    <t>CB LITE ORD</t>
-  </si>
-  <si>
-    <t>CBC 4.4 NCP</t>
-  </si>
-  <si>
-    <t>CB Original NCP</t>
-  </si>
-  <si>
-    <t>CB LITE NCP</t>
-  </si>
-  <si>
-    <t>CB BLACK NCP</t>
-  </si>
-  <si>
-    <t>CAMBODIA COLA</t>
+    <t>No Compromise</t>
+  </si>
+  <si>
+    <t>4. របាយការណ៍លក់ជូនអតិថិជនមិនពិត (ទាំងចំនួនលក់ និងតម្លៃ)។</t>
+  </si>
+  <si>
+    <t>បញ្ហាទីផ្សារ</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> បញ្ហាត្រូវដោះស្រាយ</t>
+  </si>
+  <si>
+    <t>1.Mass Products មិនត្រូវឲ្យខ្វះស្លកក្នុងផ្ទះមួយ(CBL/Wurkz/Exprez/Dazz/Water/Sport PET 500ml/Ize PET 500ml)</t>
+  </si>
+  <si>
+    <t>2.ផលិតផលហួសការកំណត់</t>
+  </si>
+  <si>
+    <t>3. ការបញ្ចូលរបាយការណ៍លក់មិនត្រឹមត្រូវ</t>
   </si>
   <si>
     <t>WURKZ ORD</t>
   </si>
   <si>
+    <t>Wurkz Ice ORD</t>
+  </si>
+  <si>
+    <t>CAMBODIA ED ORD</t>
+  </si>
+  <si>
     <t>DAZZ ORD</t>
   </si>
   <si>
-    <t>IZE PET 300ml Flavour</t>
-  </si>
-  <si>
-    <t>IZE COLA PET 1.5L All SKUs</t>
+    <t>DAZZ Zero Sugar ORD</t>
   </si>
   <si>
     <t>EXPREZ Melon ORD</t>
   </si>
   <si>
+    <t>CAMBODIA Sport 500ml ORD</t>
+  </si>
+  <si>
     <t>EXPREZ Can 330ml ORD</t>
   </si>
   <si>
-    <t>Wurkz Ice ORD</t>
-  </si>
-  <si>
-    <t>CAMBODIA Sport 500ml ORD</t>
-  </si>
-  <si>
-    <t>CAMBODIA WATER 500mL</t>
-  </si>
-  <si>
-    <t>CAMBODIA WATER 1500mL</t>
-  </si>
-  <si>
-    <t>PRODUCT MOVEMENT VS COMPETITOR</t>
-  </si>
-  <si>
-    <t>#</t>
-  </si>
-  <si>
-    <t>Mov</t>
-  </si>
-  <si>
-    <t>Stock</t>
-  </si>
-  <si>
-    <t>Buy In</t>
-  </si>
-  <si>
-    <t>Sell Out</t>
-  </si>
-  <si>
-    <t>Ring Pull</t>
-  </si>
-  <si>
-    <t>GB SNOW ORD</t>
-  </si>
-  <si>
-    <t>HANUMAN LITE ORD</t>
-  </si>
-  <si>
-    <t>Krud LITE ORD</t>
-  </si>
-  <si>
-    <t>GB Original NCP</t>
-  </si>
-  <si>
-    <t>Krud NCP</t>
-  </si>
-  <si>
-    <t>GB SNOW NCP</t>
-  </si>
-  <si>
-    <t>Hanuman LITE NCP</t>
-  </si>
-  <si>
-    <t>Krud LITE NCP</t>
-  </si>
-  <si>
-    <t>Greet LITE NCP</t>
-  </si>
-  <si>
-    <t>Hanuman Black NCP</t>
-  </si>
-  <si>
-    <t>CAMBODIA COLA 330ml</t>
-  </si>
-  <si>
-    <t>Coca Cola 330ml</t>
+    <t>Idol Can 330ml ORD</t>
   </si>
   <si>
     <t>Boostrong ORD</t>
@@ -190,106 +298,16 @@
     <t>Krud Ice ORD</t>
   </si>
   <si>
-    <t>CAMBODIA ED ORD</t>
+    <t>King Kong ORD</t>
   </si>
   <si>
     <t>Super Boostrong ORD</t>
   </si>
   <si>
-    <t>King Kong ORD</t>
-  </si>
-  <si>
     <t xml:space="preserve">AIRA </t>
   </si>
   <si>
     <t>Dragon ORD</t>
-  </si>
-  <si>
-    <t>BACCHUSE Sugar Free</t>
-  </si>
-  <si>
-    <t>IZE PET 300ml All SKUs</t>
-  </si>
-  <si>
-    <t>POP Z Flavour</t>
-  </si>
-  <si>
-    <t>V Cola 350ml</t>
-  </si>
-  <si>
-    <t>Coca 1.5L</t>
-  </si>
-  <si>
-    <t>Big Cola 3L</t>
-  </si>
-  <si>
-    <t>Sting Can 330ml</t>
-  </si>
-  <si>
-    <t>Idol Can 330ml ORD</t>
-  </si>
-  <si>
-    <t>Pocari Sweat</t>
-  </si>
-  <si>
-    <t>V-Active Sport</t>
-  </si>
-  <si>
-    <t>Vital 500mL</t>
-  </si>
-  <si>
-    <t>Provida 500mL</t>
-  </si>
-  <si>
-    <t>Ganzberg 500ml</t>
-  </si>
-  <si>
-    <t>Hitech 500mL</t>
-  </si>
-  <si>
-    <t>Vital 1500mL</t>
-  </si>
-  <si>
-    <t>Provida 1500mL</t>
-  </si>
-  <si>
-    <t>Ganzberg 1500ml</t>
-  </si>
-  <si>
-    <t>Hitech 1500mL</t>
-  </si>
-  <si>
-    <t>No Compromise</t>
-  </si>
-  <si>
-    <t>បញ្ហាទីផ្សារ</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> បញ្ហាត្រូវដោះស្រាយ</t>
-  </si>
-  <si>
-    <t>1.Mass Products មិនត្រូវឲ្យខ្វះស្លកក្នុងផ្ទះមួយ(CBL/Wurkz/Exprez/Dazz/Water/Sport PET 500ml/Ize PET 500ml)</t>
-  </si>
-  <si>
-    <t>2.ផលិតផលហួសការកំណត់</t>
-  </si>
-  <si>
-    <t>2.</t>
-  </si>
-  <si>
-    <t>3. ការបញ្ចូលរបាយការណ៍លក់មិនត្រឹមត្រូវ</t>
-  </si>
-  <si>
-    <t>3.</t>
-  </si>
-  <si>
-    <t>4. របាយការណ៍លក់ជូនអតិថិជនមិនពិត (ទាំងចំនួនលក់ និងតម្លៃ)។</t>
-  </si>
-  <si>
-    <t>4.</t>
-  </si>
-  <si>
-    <t>DAZZ Zero Sugar ORD</t>
   </si>
   <si>
     <t>BACCHUSE</t>
@@ -299,7 +317,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -352,32 +370,58 @@
       <b/>
       <sz val="18"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="18"/>
       <name val="Noto Sans Khmer"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="28"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="18"/>
       <color rgb="FFFFFFFF"/>
       <name val="Noto Sans Khmer"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="18"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="18"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="16.0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="16.0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="16.0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="16.0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -405,6 +449,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -490,7 +535,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -572,6 +617,18 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -601,19 +658,17 @@
     <xdr:ext cx="1047750" cy="1047750"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="/xl/media/image.png">
+        <xdr:cNvPr id="2" name="Image 1" descr="Picture">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
+        <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -641,27 +696,48 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="/xl/media/image2.png">
+        <xdr:cNvPr id="1025" name="Image 1" descr="Picture">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C0AC80C4-2B8A-06F4-AB2F-4BE414DA6D6E}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
-      <xdr:spPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1047750" cy="1047750"/>
+        </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -681,27 +757,48 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="/xl/media/image2.png">
+        <xdr:cNvPr id="1026" name="Picture 2" descr="Picture">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{95199885-0DDC-586F-4B36-11B1346C57DC}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
-      <xdr:spPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1047750" cy="1047750"/>
+        </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -721,27 +818,48 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="/xl/media/image2.png">
+        <xdr:cNvPr id="3" name="Image 1" descr="Picture">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000005000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F4978D84-8A64-D7B4-F157-6A10E3767AF3}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
-      <xdr:spPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1047750" cy="1047750"/>
+        </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -761,27 +879,48 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="/xl/media/image2.png">
+        <xdr:cNvPr id="4" name="Picture 2" descr="Picture">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000006000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1F87ED97-C3A1-E2C8-2CA7-4111409C6EC9}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
-      <xdr:spPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1047750" cy="1047750"/>
+        </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -801,27 +940,48 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="/xl/media/image2.png">
+        <xdr:cNvPr id="1027" name="Picture 3" descr="Picture">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000007000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6C034566-D112-44CE-AE72-A84C420E2B15}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
+          <a:picLocks noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
-      <xdr:spPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1047750" cy="1047750"/>
+        </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -1045,6 +1205,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:AA49"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1066,11 +1229,11 @@
     <col min="26" max="27" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" ht="54.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:27" ht="82" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="4"/>
       <c r="D1" s="5"/>
     </row>
-    <row r="2" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="29" t="s">
         <v>0</v>
       </c>
@@ -1101,9 +1264,9 @@
       <c r="Z2" s="12"/>
       <c r="AA2" s="12"/>
     </row>
-    <row r="3" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="11" t="s">
-        <v>1</v>
+        <v>65</v>
       </c>
       <c r="B3" s="12"/>
       <c r="C3" s="12"/>
@@ -1132,20 +1295,20 @@
       <c r="Z3" s="12"/>
       <c r="AA3" s="12"/>
     </row>
-    <row r="4" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A4" s="20" t="s">
-        <v>2</v>
+        <v>62</v>
       </c>
       <c r="B4" s="15"/>
       <c r="C4" s="20" t="s">
-        <v>3</v>
+        <v>63</v>
       </c>
       <c r="D4" s="14"/>
       <c r="E4" s="14"/>
       <c r="F4" s="14"/>
       <c r="G4" s="15"/>
       <c r="H4" s="28" t="s">
-        <v>4</v>
+        <v>61</v>
       </c>
       <c r="I4" s="14"/>
       <c r="J4" s="14"/>
@@ -1162,16 +1325,16 @@
       <c r="U4" s="14"/>
       <c r="V4" s="15"/>
       <c r="W4" s="20" t="s">
-        <v>5</v>
+        <v>64</v>
       </c>
       <c r="X4" s="14"/>
       <c r="Y4" s="14"/>
       <c r="Z4" s="14"/>
       <c r="AA4" s="15"/>
     </row>
-    <row r="5" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="18" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B5" s="14"/>
       <c r="C5" s="14"/>
@@ -1200,59 +1363,59 @@
       <c r="Z5" s="14"/>
       <c r="AA5" s="15"/>
     </row>
-    <row r="6" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C6" s="22" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D6" s="14"/>
       <c r="E6" s="14"/>
       <c r="F6" s="14"/>
       <c r="G6" s="15"/>
       <c r="H6" s="19" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I6" s="14"/>
       <c r="J6" s="14"/>
       <c r="K6" s="15"/>
       <c r="L6" s="19" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="M6" s="14"/>
       <c r="N6" s="14"/>
       <c r="O6" s="15"/>
       <c r="P6" s="19" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="Q6" s="14"/>
       <c r="R6" s="14"/>
       <c r="S6" s="15"/>
       <c r="T6" s="19" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="U6" s="14"/>
       <c r="V6" s="15"/>
       <c r="W6" s="21" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="X6" s="14"/>
       <c r="Y6" s="15"/>
       <c r="Z6" s="21" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="AA6" s="15"/>
     </row>
-    <row r="7" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
         <v>1</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C7" s="13"/>
       <c r="D7" s="14"/>
@@ -1290,12 +1453,12 @@
       <c r="Z7" s="13"/>
       <c r="AA7" s="15"/>
     </row>
-    <row r="8" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
         <v>2</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C8" s="13"/>
       <c r="D8" s="14"/>
@@ -1333,12 +1496,12 @@
       <c r="Z8" s="13"/>
       <c r="AA8" s="15"/>
     </row>
-    <row r="9" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
         <v>3</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="C9" s="13"/>
       <c r="D9" s="14"/>
@@ -1376,12 +1539,12 @@
       <c r="Z9" s="13"/>
       <c r="AA9" s="15"/>
     </row>
-    <row r="10" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3">
         <v>4</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="C10" s="13"/>
       <c r="D10" s="14"/>
@@ -1419,12 +1582,12 @@
       <c r="Z10" s="13"/>
       <c r="AA10" s="15"/>
     </row>
-    <row r="11" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
         <v>5</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C11" s="13"/>
       <c r="D11" s="14"/>
@@ -1462,12 +1625,12 @@
       <c r="Z11" s="13"/>
       <c r="AA11" s="15"/>
     </row>
-    <row r="12" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3">
         <v>6</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="C12" s="13"/>
       <c r="D12" s="14"/>
@@ -1505,12 +1668,12 @@
       <c r="Z12" s="13"/>
       <c r="AA12" s="15"/>
     </row>
-    <row r="13" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="3">
         <v>7</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>22</v>
+        <v>73</v>
       </c>
       <c r="C13" s="13"/>
       <c r="D13" s="14"/>
@@ -1548,12 +1711,12 @@
       <c r="Z13" s="13"/>
       <c r="AA13" s="15"/>
     </row>
-    <row r="14" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3">
         <v>8</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="C14" s="13"/>
       <c r="D14" s="14"/>
@@ -1591,12 +1754,12 @@
       <c r="Z14" s="13"/>
       <c r="AA14" s="15"/>
     </row>
-    <row r="15" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="3">
         <v>9</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>23</v>
+        <v>76</v>
       </c>
       <c r="C15" s="13"/>
       <c r="D15" s="14"/>
@@ -1634,12 +1797,12 @@
       <c r="Z15" s="13"/>
       <c r="AA15" s="15"/>
     </row>
-    <row r="16" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3">
         <v>10</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="C16" s="13"/>
       <c r="D16" s="14"/>
@@ -1677,12 +1840,12 @@
       <c r="Z16" s="13"/>
       <c r="AA16" s="15"/>
     </row>
-    <row r="17" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="3">
         <v>11</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C17" s="13"/>
       <c r="D17" s="14"/>
@@ -1720,12 +1883,12 @@
       <c r="Z17" s="13"/>
       <c r="AA17" s="15"/>
     </row>
-    <row r="18" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="3">
         <v>12</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="C18" s="13"/>
       <c r="D18" s="14"/>
@@ -1763,12 +1926,12 @@
       <c r="Z18" s="13"/>
       <c r="AA18" s="15"/>
     </row>
-    <row r="19" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="3">
         <v>13</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>26</v>
+        <v>78</v>
       </c>
       <c r="C19" s="13"/>
       <c r="D19" s="14"/>
@@ -1806,12 +1969,12 @@
       <c r="Z19" s="13"/>
       <c r="AA19" s="15"/>
     </row>
-    <row r="20" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="3">
         <v>14</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>27</v>
+        <v>80</v>
       </c>
       <c r="C20" s="13"/>
       <c r="D20" s="14"/>
@@ -1849,12 +2012,12 @@
       <c r="Z20" s="13"/>
       <c r="AA20" s="15"/>
     </row>
-    <row r="21" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A21" s="3">
         <v>15</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>28</v>
+        <v>74</v>
       </c>
       <c r="C21" s="13"/>
       <c r="D21" s="14"/>
@@ -1892,12 +2055,12 @@
       <c r="Z21" s="13"/>
       <c r="AA21" s="15"/>
     </row>
-    <row r="22" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="3">
         <v>16</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>29</v>
+        <v>79</v>
       </c>
       <c r="C22" s="13"/>
       <c r="D22" s="14"/>
@@ -1935,12 +2098,12 @@
       <c r="Z22" s="13"/>
       <c r="AA22" s="15"/>
     </row>
-    <row r="23" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="3">
         <v>17</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C23" s="13"/>
       <c r="D23" s="14"/>
@@ -1978,12 +2141,12 @@
       <c r="Z23" s="13"/>
       <c r="AA23" s="15"/>
     </row>
-    <row r="24" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="3">
         <v>18</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="C24" s="13"/>
       <c r="D24" s="14"/>
@@ -2021,9 +2184,9 @@
       <c r="Z24" s="13"/>
       <c r="AA24" s="15"/>
     </row>
-    <row r="25" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="24" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="12"/>
@@ -2052,95 +2215,95 @@
       <c r="Z25" s="12"/>
       <c r="AA25" s="12"/>
     </row>
-    <row r="26" spans="1:27" ht="12" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:27" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="6" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I26" s="6" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="J26" s="6" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="K26" s="6" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="L26" s="6" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="M26" s="6" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="N26" s="6" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="O26" s="6" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="P26" s="6" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="Q26" s="6" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="R26" s="6" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="S26" s="6" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="T26" s="6" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="U26" s="6" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="V26" s="6" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="W26" s="6" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="X26" s="6" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="Y26" s="6" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="Z26" s="6" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="AA26" s="6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="27" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="27" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="3">
         <v>1</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C27" s="3"/>
       <c r="D27" s="7"/>
@@ -2148,21 +2311,21 @@
       <c r="F27" s="8"/>
       <c r="G27" s="3"/>
       <c r="H27" s="1" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="I27" s="3"/>
       <c r="J27" s="3"/>
       <c r="K27" s="3"/>
       <c r="L27" s="3"/>
       <c r="M27" s="1" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="N27" s="3"/>
       <c r="O27" s="3"/>
       <c r="P27" s="3"/>
       <c r="Q27" s="3"/>
       <c r="R27" s="1" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="S27" s="3"/>
       <c r="T27" s="3"/>
@@ -2174,12 +2337,12 @@
       <c r="Z27" s="3"/>
       <c r="AA27" s="3"/>
     </row>
-    <row r="28" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="3">
         <v>2</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C28" s="3"/>
       <c r="D28" s="7"/>
@@ -2187,21 +2350,21 @@
       <c r="F28" s="8"/>
       <c r="G28" s="8"/>
       <c r="H28" s="1" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="I28" s="3"/>
       <c r="J28" s="7"/>
       <c r="K28" s="8"/>
       <c r="L28" s="8"/>
       <c r="M28" s="1" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="N28" s="3"/>
       <c r="O28" s="3"/>
       <c r="P28" s="3"/>
       <c r="Q28" s="3"/>
       <c r="R28" s="1" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="S28" s="3"/>
       <c r="T28" s="3"/>
@@ -2213,12 +2376,12 @@
       <c r="Z28" s="3"/>
       <c r="AA28" s="3"/>
     </row>
-    <row r="29" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="3">
         <v>3</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="C29" s="3"/>
       <c r="D29" s="7"/>
@@ -2226,40 +2389,40 @@
       <c r="F29" s="8"/>
       <c r="G29" s="8"/>
       <c r="H29" s="1" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="I29" s="3"/>
       <c r="J29" s="3"/>
       <c r="K29" s="3"/>
       <c r="L29" s="3"/>
       <c r="M29" s="1" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="N29" s="3"/>
       <c r="O29" s="3"/>
       <c r="P29" s="3"/>
       <c r="Q29" s="3"/>
       <c r="R29" s="1" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="S29" s="3"/>
       <c r="T29" s="3"/>
       <c r="U29" s="3"/>
       <c r="V29" s="3"/>
       <c r="W29" s="1" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="X29" s="3"/>
       <c r="Y29" s="3"/>
       <c r="Z29" s="3"/>
       <c r="AA29" s="3"/>
     </row>
-    <row r="30" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="3">
         <v>4</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
@@ -2272,7 +2435,7 @@
       <c r="K30" s="3"/>
       <c r="L30" s="3"/>
       <c r="M30" s="1" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="N30" s="3"/>
       <c r="O30" s="3"/>
@@ -2289,12 +2452,12 @@
       <c r="Z30" s="3"/>
       <c r="AA30" s="3"/>
     </row>
-    <row r="31" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="3">
         <v>5</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
@@ -2302,7 +2465,7 @@
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
       <c r="H31" s="1" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="I31" s="3"/>
       <c r="J31" s="3"/>
@@ -2324,12 +2487,12 @@
       <c r="Z31" s="3"/>
       <c r="AA31" s="3"/>
     </row>
-    <row r="32" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="3">
         <v>6</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>22</v>
+        <v>73</v>
       </c>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
@@ -2337,7 +2500,7 @@
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
       <c r="H32" s="1" t="s">
-        <v>51</v>
+        <v>82</v>
       </c>
       <c r="I32" s="3"/>
       <c r="J32" s="3"/>
@@ -2349,7 +2512,7 @@
       <c r="P32" s="3"/>
       <c r="Q32" s="3"/>
       <c r="R32" s="1" t="s">
-        <v>52</v>
+        <v>83</v>
       </c>
       <c r="S32" s="3"/>
       <c r="T32" s="3"/>
@@ -2361,12 +2524,12 @@
       <c r="Z32" s="3"/>
       <c r="AA32" s="3"/>
     </row>
-    <row r="33" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="3">
         <v>7</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>28</v>
+        <v>74</v>
       </c>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
@@ -2374,21 +2537,21 @@
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
       <c r="H33" s="1" t="s">
-        <v>53</v>
+        <v>84</v>
       </c>
       <c r="I33" s="3"/>
       <c r="J33" s="3"/>
       <c r="K33" s="3"/>
       <c r="L33" s="3"/>
       <c r="M33" s="1" t="s">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="N33" s="3"/>
       <c r="O33" s="3"/>
       <c r="P33" s="3"/>
       <c r="Q33" s="3"/>
       <c r="R33" s="1" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="S33" s="3"/>
       <c r="T33" s="3"/>
@@ -2400,12 +2563,12 @@
       <c r="Z33" s="3"/>
       <c r="AA33" s="3"/>
     </row>
-    <row r="34" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="3">
         <v>8</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="C34" s="3"/>
       <c r="D34" s="7"/>
@@ -2413,21 +2576,21 @@
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
       <c r="H34" s="1" t="s">
-        <v>57</v>
+        <v>88</v>
       </c>
       <c r="I34" s="3"/>
       <c r="J34" s="3"/>
       <c r="K34" s="3"/>
       <c r="L34" s="3"/>
       <c r="M34" s="1" t="s">
-        <v>58</v>
+        <v>87</v>
       </c>
       <c r="N34" s="3"/>
       <c r="O34" s="3"/>
       <c r="P34" s="3"/>
       <c r="Q34" s="3"/>
       <c r="R34" s="1" t="s">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="S34" s="3"/>
       <c r="T34" s="3"/>
@@ -2439,12 +2602,12 @@
       <c r="Z34" s="3"/>
       <c r="AA34" s="3"/>
     </row>
-    <row r="35" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="3">
         <v>9</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>23</v>
+        <v>76</v>
       </c>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
@@ -2452,7 +2615,7 @@
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
       <c r="H35" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I35" s="3"/>
       <c r="J35" s="3"/>
@@ -2464,7 +2627,7 @@
       <c r="P35" s="3"/>
       <c r="Q35" s="3"/>
       <c r="R35" s="1" t="s">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="S35" s="3"/>
       <c r="T35" s="3"/>
@@ -2476,12 +2639,12 @@
       <c r="Z35" s="3"/>
       <c r="AA35" s="3"/>
     </row>
-    <row r="36" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="3">
         <v>10</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
@@ -2489,7 +2652,7 @@
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
       <c r="H36" s="1" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="I36" s="3"/>
       <c r="J36" s="3"/>
@@ -2511,12 +2674,12 @@
       <c r="Z36" s="3"/>
       <c r="AA36" s="3"/>
     </row>
-    <row r="37" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="3">
         <v>11</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>62</v>
+        <v>42</v>
       </c>
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
@@ -2524,7 +2687,7 @@
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
       <c r="H37" s="1" t="s">
-        <v>63</v>
+        <v>43</v>
       </c>
       <c r="I37" s="3"/>
       <c r="J37" s="3"/>
@@ -2536,7 +2699,7 @@
       <c r="P37" s="3"/>
       <c r="Q37" s="3"/>
       <c r="R37" s="1" t="s">
-        <v>64</v>
+        <v>44</v>
       </c>
       <c r="S37" s="3"/>
       <c r="T37" s="3"/>
@@ -2548,12 +2711,12 @@
       <c r="Z37" s="3"/>
       <c r="AA37" s="3"/>
     </row>
-    <row r="38" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="3">
         <v>12</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="C38" s="3"/>
       <c r="D38" s="3"/>
@@ -2561,14 +2724,14 @@
       <c r="F38" s="3"/>
       <c r="G38" s="3"/>
       <c r="H38" s="1" t="s">
-        <v>65</v>
+        <v>45</v>
       </c>
       <c r="I38" s="3"/>
       <c r="J38" s="3"/>
       <c r="K38" s="3"/>
       <c r="L38" s="3"/>
       <c r="M38" s="1" t="s">
-        <v>66</v>
+        <v>46</v>
       </c>
       <c r="N38" s="3"/>
       <c r="O38" s="3"/>
@@ -2585,12 +2748,12 @@
       <c r="Z38" s="3"/>
       <c r="AA38" s="3"/>
     </row>
-    <row r="39" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="3">
         <v>13</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>26</v>
+        <v>78</v>
       </c>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
@@ -2598,21 +2761,21 @@
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
       <c r="H39" s="1" t="s">
-        <v>27</v>
+        <v>80</v>
       </c>
       <c r="I39" s="3"/>
       <c r="J39" s="3"/>
       <c r="K39" s="3"/>
       <c r="L39" s="3"/>
       <c r="M39" s="1" t="s">
-        <v>67</v>
+        <v>47</v>
       </c>
       <c r="N39" s="3"/>
       <c r="O39" s="3"/>
       <c r="P39" s="3"/>
       <c r="Q39" s="3"/>
       <c r="R39" s="1" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="S39" s="3"/>
       <c r="T39" s="3"/>
@@ -2624,12 +2787,12 @@
       <c r="Z39" s="3"/>
       <c r="AA39" s="3"/>
     </row>
-    <row r="40" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="3">
         <v>14</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>29</v>
+        <v>79</v>
       </c>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
@@ -2642,14 +2805,14 @@
       <c r="K40" s="3"/>
       <c r="L40" s="3"/>
       <c r="M40" s="1" t="s">
-        <v>69</v>
+        <v>48</v>
       </c>
       <c r="N40" s="3"/>
       <c r="O40" s="3"/>
       <c r="P40" s="3"/>
       <c r="Q40" s="3"/>
       <c r="R40" s="1" t="s">
-        <v>70</v>
+        <v>49</v>
       </c>
       <c r="S40" s="3"/>
       <c r="T40" s="3"/>
@@ -2661,12 +2824,12 @@
       <c r="Z40" s="3"/>
       <c r="AA40" s="3"/>
     </row>
-    <row r="41" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="3">
         <v>15</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C41" s="3"/>
       <c r="D41" s="3"/>
@@ -2674,40 +2837,40 @@
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
       <c r="H41" s="1" t="s">
-        <v>71</v>
+        <v>50</v>
       </c>
       <c r="I41" s="3"/>
       <c r="J41" s="3"/>
       <c r="K41" s="3"/>
       <c r="L41" s="3"/>
       <c r="M41" s="1" t="s">
-        <v>72</v>
+        <v>51</v>
       </c>
       <c r="N41" s="3"/>
       <c r="O41" s="3"/>
       <c r="P41" s="3"/>
       <c r="Q41" s="3"/>
       <c r="R41" s="1" t="s">
-        <v>73</v>
+        <v>52</v>
       </c>
       <c r="S41" s="3"/>
       <c r="T41" s="3"/>
       <c r="U41" s="3"/>
       <c r="V41" s="3"/>
       <c r="W41" s="1" t="s">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="X41" s="3"/>
       <c r="Y41" s="3"/>
       <c r="Z41" s="3"/>
       <c r="AA41" s="3"/>
     </row>
-    <row r="42" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A42" s="3">
         <v>16</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="C42" s="3"/>
       <c r="D42" s="3"/>
@@ -2715,35 +2878,35 @@
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
       <c r="H42" s="1" t="s">
-        <v>75</v>
+        <v>54</v>
       </c>
       <c r="I42" s="3"/>
       <c r="J42" s="3"/>
       <c r="K42" s="3"/>
       <c r="L42" s="3"/>
       <c r="M42" s="1" t="s">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="N42" s="3"/>
       <c r="O42" s="3"/>
       <c r="P42" s="3"/>
       <c r="Q42" s="3"/>
       <c r="R42" s="1" t="s">
-        <v>77</v>
+        <v>56</v>
       </c>
       <c r="S42" s="3"/>
       <c r="T42" s="3"/>
       <c r="U42" s="3"/>
       <c r="V42" s="3"/>
       <c r="W42" s="1" t="s">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="X42" s="3"/>
       <c r="Y42" s="3"/>
       <c r="Z42" s="3"/>
       <c r="AA42" s="3"/>
     </row>
-    <row r="43" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="9"/>
       <c r="B43" s="9"/>
       <c r="C43" s="9"/>
@@ -2752,9 +2915,9 @@
       <c r="F43" s="9"/>
       <c r="G43" s="9"/>
     </row>
-    <row r="44" spans="1:27" ht="26.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:27" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="27" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="B44" s="27"/>
       <c r="C44" s="27"/>
@@ -2764,7 +2927,7 @@
       <c r="G44" s="27"/>
       <c r="H44" s="10"/>
       <c r="I44" s="17" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="J44" s="30"/>
       <c r="K44" s="30"/>
@@ -2775,7 +2938,7 @@
       <c r="P44" s="30"/>
       <c r="Q44" s="30"/>
       <c r="S44" s="17" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="T44" s="12"/>
       <c r="U44" s="12"/>
@@ -2786,9 +2949,9 @@
       <c r="Z44" s="12"/>
       <c r="AA44" s="12"/>
     </row>
-    <row r="45" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="25" t="s">
-        <v>82</v>
+    <row r="45" spans="1:27" ht="54" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="31" t="s">
+        <v>70</v>
       </c>
       <c r="B45" s="23"/>
       <c r="C45" s="23"/>
@@ -2819,9 +2982,9 @@
       <c r="Z45" s="12"/>
       <c r="AA45" s="12"/>
     </row>
-    <row r="46" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="23" t="s">
-        <v>83</v>
+    <row r="46" spans="1:27" ht="54" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="32" t="s">
+        <v>71</v>
       </c>
       <c r="B46" s="23"/>
       <c r="C46" s="23"/>
@@ -2830,7 +2993,7 @@
       <c r="F46" s="23"/>
       <c r="G46" s="23"/>
       <c r="I46" s="16" t="s">
-        <v>84</v>
+        <v>58</v>
       </c>
       <c r="J46" s="16"/>
       <c r="K46" s="16"/>
@@ -2841,7 +3004,7 @@
       <c r="P46" s="16"/>
       <c r="Q46" s="16"/>
       <c r="S46" s="16" t="s">
-        <v>84</v>
+        <v>58</v>
       </c>
       <c r="T46" s="12"/>
       <c r="U46" s="12"/>
@@ -2852,9 +3015,9 @@
       <c r="Z46" s="12"/>
       <c r="AA46" s="12"/>
     </row>
-    <row r="47" spans="1:27" ht="36" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="23" t="s">
-        <v>85</v>
+    <row r="47" spans="1:27" ht="54" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="33" t="s">
+        <v>72</v>
       </c>
       <c r="B47" s="24"/>
       <c r="C47" s="24"/>
@@ -2863,7 +3026,7 @@
       <c r="F47" s="24"/>
       <c r="G47" s="24"/>
       <c r="I47" s="16" t="s">
-        <v>86</v>
+        <v>59</v>
       </c>
       <c r="J47" s="16"/>
       <c r="K47" s="16"/>
@@ -2874,7 +3037,7 @@
       <c r="P47" s="16"/>
       <c r="Q47" s="16"/>
       <c r="S47" s="16" t="s">
-        <v>86</v>
+        <v>59</v>
       </c>
       <c r="T47" s="12"/>
       <c r="U47" s="12"/>
@@ -2885,9 +3048,9 @@
       <c r="Z47" s="12"/>
       <c r="AA47" s="12"/>
     </row>
-    <row r="48" spans="1:27" ht="33.4" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="23" t="s">
-        <v>87</v>
+    <row r="48" spans="1:27" ht="50" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A48" s="34" t="s">
+        <v>67</v>
       </c>
       <c r="B48" s="24"/>
       <c r="C48" s="24"/>
@@ -2896,7 +3059,7 @@
       <c r="F48" s="24"/>
       <c r="G48" s="24"/>
       <c r="I48" s="16" t="s">
-        <v>88</v>
+        <v>60</v>
       </c>
       <c r="J48" s="16"/>
       <c r="K48" s="16"/>
@@ -2907,7 +3070,7 @@
       <c r="P48" s="16"/>
       <c r="Q48" s="16"/>
       <c r="S48" s="16" t="s">
-        <v>88</v>
+        <v>60</v>
       </c>
       <c r="T48" s="12"/>
       <c r="U48" s="12"/>
@@ -2918,11 +3081,9 @@
       <c r="Z48" s="12"/>
       <c r="AA48" s="12"/>
     </row>
-    <row r="49" ht="16.649999999999999" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="49" ht="25" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <mergeCells count="156">
-    <mergeCell ref="W7:Y7"/>
-    <mergeCell ref="C12:G12"/>
     <mergeCell ref="S48:AA48"/>
     <mergeCell ref="W16:Y16"/>
     <mergeCell ref="I45:Q45"/>
@@ -2937,12 +3098,16 @@
     <mergeCell ref="H24:K24"/>
     <mergeCell ref="I44:Q44"/>
     <mergeCell ref="I46:Q46"/>
+    <mergeCell ref="P13:S13"/>
+    <mergeCell ref="Z10:AA10"/>
     <mergeCell ref="A2:AA2"/>
     <mergeCell ref="W18:Y18"/>
     <mergeCell ref="P20:S20"/>
     <mergeCell ref="W8:Y8"/>
     <mergeCell ref="T6:V6"/>
+    <mergeCell ref="Z21:AA21"/>
     <mergeCell ref="L19:O19"/>
+    <mergeCell ref="C21:G21"/>
     <mergeCell ref="H9:K9"/>
     <mergeCell ref="L12:O12"/>
     <mergeCell ref="P6:S6"/>
@@ -2953,6 +3118,17 @@
     <mergeCell ref="T14:V14"/>
     <mergeCell ref="P18:S18"/>
     <mergeCell ref="Z11:AA11"/>
+    <mergeCell ref="C14:G14"/>
+    <mergeCell ref="W7:Y7"/>
+    <mergeCell ref="C12:G12"/>
+    <mergeCell ref="A47:G47"/>
+    <mergeCell ref="L17:O17"/>
+    <mergeCell ref="Z22:AA22"/>
+    <mergeCell ref="C22:G22"/>
+    <mergeCell ref="S46:AA46"/>
+    <mergeCell ref="H23:K23"/>
+    <mergeCell ref="A44:G44"/>
+    <mergeCell ref="Z19:AA19"/>
     <mergeCell ref="H4:V4"/>
     <mergeCell ref="C18:G18"/>
     <mergeCell ref="S47:AA47"/>
@@ -2969,68 +3145,68 @@
     <mergeCell ref="Z24:AA24"/>
     <mergeCell ref="C20:G20"/>
     <mergeCell ref="C4:G4"/>
-    <mergeCell ref="A47:G47"/>
-    <mergeCell ref="L17:O17"/>
-    <mergeCell ref="Z22:AA22"/>
-    <mergeCell ref="C22:G22"/>
-    <mergeCell ref="S46:AA46"/>
-    <mergeCell ref="H23:K23"/>
-    <mergeCell ref="A44:G44"/>
-    <mergeCell ref="Z19:AA19"/>
-    <mergeCell ref="Z21:AA21"/>
-    <mergeCell ref="C21:G21"/>
-    <mergeCell ref="H11:K11"/>
-    <mergeCell ref="L20:O20"/>
-    <mergeCell ref="H8:K8"/>
-    <mergeCell ref="W9:Y9"/>
-    <mergeCell ref="T8:V8"/>
-    <mergeCell ref="T17:V17"/>
-    <mergeCell ref="L16:O16"/>
-    <mergeCell ref="P9:S9"/>
-    <mergeCell ref="P13:S13"/>
-    <mergeCell ref="Z8:AA8"/>
-    <mergeCell ref="W14:Y14"/>
-    <mergeCell ref="Z17:AA17"/>
-    <mergeCell ref="W22:Y22"/>
-    <mergeCell ref="W13:Y13"/>
-    <mergeCell ref="Z9:AA9"/>
-    <mergeCell ref="Z14:AA14"/>
-    <mergeCell ref="W10:Y10"/>
-    <mergeCell ref="Z10:AA10"/>
-    <mergeCell ref="C10:G10"/>
     <mergeCell ref="I48:Q48"/>
     <mergeCell ref="P17:S17"/>
     <mergeCell ref="H16:K16"/>
     <mergeCell ref="L10:O10"/>
     <mergeCell ref="C13:G13"/>
     <mergeCell ref="L24:O24"/>
+    <mergeCell ref="T24:V24"/>
     <mergeCell ref="P19:S19"/>
     <mergeCell ref="C15:G15"/>
     <mergeCell ref="P12:S12"/>
     <mergeCell ref="C16:G16"/>
+    <mergeCell ref="T22:V22"/>
     <mergeCell ref="C24:G24"/>
     <mergeCell ref="A48:G48"/>
+    <mergeCell ref="T16:V16"/>
     <mergeCell ref="A45:G45"/>
+    <mergeCell ref="T13:V13"/>
     <mergeCell ref="A46:G46"/>
     <mergeCell ref="P11:S11"/>
+    <mergeCell ref="H17:K17"/>
+    <mergeCell ref="H11:K11"/>
+    <mergeCell ref="L20:O20"/>
+    <mergeCell ref="T17:V17"/>
+    <mergeCell ref="L16:O16"/>
     <mergeCell ref="W24:Y24"/>
     <mergeCell ref="L22:O22"/>
     <mergeCell ref="P22:S22"/>
     <mergeCell ref="C23:G23"/>
     <mergeCell ref="H12:K12"/>
+    <mergeCell ref="L6:O6"/>
     <mergeCell ref="T12:V12"/>
     <mergeCell ref="T21:V21"/>
     <mergeCell ref="P15:S15"/>
     <mergeCell ref="H14:K14"/>
-    <mergeCell ref="T24:V24"/>
-    <mergeCell ref="T22:V22"/>
-    <mergeCell ref="T16:V16"/>
-    <mergeCell ref="T13:V13"/>
+    <mergeCell ref="C10:G10"/>
+    <mergeCell ref="W14:Y14"/>
+    <mergeCell ref="W22:Y22"/>
+    <mergeCell ref="W13:Y13"/>
+    <mergeCell ref="W10:Y10"/>
     <mergeCell ref="W23:Y23"/>
-    <mergeCell ref="H17:K17"/>
-    <mergeCell ref="C14:G14"/>
-    <mergeCell ref="Z20:AA20"/>
-    <mergeCell ref="W15:Y15"/>
+    <mergeCell ref="H8:K8"/>
+    <mergeCell ref="W9:Y9"/>
+    <mergeCell ref="T8:V8"/>
+    <mergeCell ref="P9:S9"/>
+    <mergeCell ref="T10:V10"/>
+    <mergeCell ref="W4:AA4"/>
+    <mergeCell ref="H19:K19"/>
+    <mergeCell ref="Z7:AA7"/>
+    <mergeCell ref="Z16:AA16"/>
+    <mergeCell ref="Z18:AA18"/>
+    <mergeCell ref="C11:G11"/>
+    <mergeCell ref="T18:V18"/>
+    <mergeCell ref="L23:O23"/>
+    <mergeCell ref="L18:O18"/>
+    <mergeCell ref="L11:O11"/>
+    <mergeCell ref="T11:V11"/>
+    <mergeCell ref="C19:G19"/>
+    <mergeCell ref="P16:S16"/>
+    <mergeCell ref="Z8:AA8"/>
+    <mergeCell ref="Z17:AA17"/>
+    <mergeCell ref="Z9:AA9"/>
+    <mergeCell ref="Z14:AA14"/>
     <mergeCell ref="Z6:AA6"/>
     <mergeCell ref="L9:O9"/>
     <mergeCell ref="C6:G6"/>
@@ -3040,27 +3216,6 @@
     <mergeCell ref="C9:G9"/>
     <mergeCell ref="P7:S7"/>
     <mergeCell ref="H7:K7"/>
-    <mergeCell ref="T10:V10"/>
-    <mergeCell ref="H19:K19"/>
-    <mergeCell ref="Z7:AA7"/>
-    <mergeCell ref="Z16:AA16"/>
-    <mergeCell ref="Z18:AA18"/>
-    <mergeCell ref="T15:V15"/>
-    <mergeCell ref="C17:G17"/>
-    <mergeCell ref="T23:V23"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="W6:Y6"/>
-    <mergeCell ref="L8:O8"/>
-    <mergeCell ref="W4:AA4"/>
-    <mergeCell ref="C11:G11"/>
-    <mergeCell ref="T18:V18"/>
-    <mergeCell ref="L23:O23"/>
-    <mergeCell ref="L18:O18"/>
-    <mergeCell ref="L11:O11"/>
-    <mergeCell ref="T11:V11"/>
-    <mergeCell ref="C19:G19"/>
-    <mergeCell ref="P16:S16"/>
-    <mergeCell ref="L6:O6"/>
     <mergeCell ref="A3:AA3"/>
     <mergeCell ref="P14:S14"/>
     <mergeCell ref="H20:K20"/>
@@ -3077,8 +3232,17 @@
     <mergeCell ref="P8:S8"/>
     <mergeCell ref="C8:G8"/>
     <mergeCell ref="L15:O15"/>
+    <mergeCell ref="T15:V15"/>
+    <mergeCell ref="C17:G17"/>
+    <mergeCell ref="T23:V23"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="W6:Y6"/>
+    <mergeCell ref="L8:O8"/>
+    <mergeCell ref="Z20:AA20"/>
+    <mergeCell ref="W15:Y15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="landscape" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>